<commit_message>
20260512 antes de pb2022 rrhh
</commit_message>
<xml_diff>
--- a/RRHH/20260508_req18275_boton_venta_planes_colectivos/doc/Firmas Anexo Planes Grupales Abril 2026 - copia.xlsx
+++ b/RRHH/20260508_req18275_boton_venta_planes_colectivos/doc/Firmas Anexo Planes Grupales Abril 2026 - copia.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Remu2026\BUK 2026\ABRIL 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\J\RepositorioJ_github\repositorioJ\RRHH\20260508_req18275_boton_venta_planes_colectivos\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17865" windowHeight="5235"/>
   </bookViews>
   <sheets>
     <sheet name="ingresar" sheetId="2" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1354" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1122" uniqueCount="439">
   <si>
     <t>Libro: Nomina Firma Electrónica</t>
   </si>
@@ -1313,9 +1313,6 @@
   </si>
   <si>
     <t>Supervisor</t>
-  </si>
-  <si>
-    <t>Nombres</t>
   </si>
   <si>
     <t>Fecha Inicio</t>
@@ -1408,7 +1405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1420,7 +1417,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1735,18 +1731,16 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:E116"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11" style="5"/>
-    <col min="2" max="2" width="35.5" style="4" customWidth="1"/>
-    <col min="3" max="3" width="26.875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="11" style="4"/>
-    <col min="5" max="5" width="12.5" style="4" customWidth="1"/>
-    <col min="6" max="16384" width="11" style="4"/>
+    <col min="2" max="2" width="11" style="4"/>
+    <col min="3" max="3" width="12.5" style="4" customWidth="1"/>
+    <col min="4" max="16384" width="11" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>423</v>
       </c>
@@ -1754,1967 +1748,1271 @@
         <v>430</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>422</v>
-      </c>
-      <c r="D1" s="8" t="s">
         <v>431</v>
       </c>
-      <c r="E1" s="8" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="5">
         <v>96658826</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E2" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B2" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C2" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="5">
         <v>191080491</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E3" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B3" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C3" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
         <v>160180293</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E4" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B4" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C4" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="5">
         <v>131294964</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E5" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B5" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C5" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
         <v>185753204</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E6" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B6" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C6" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="5">
         <v>132361460</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E7" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B7" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C7" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="5">
         <v>168654804</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E8" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B8" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C8" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="5">
         <v>132528640</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E9" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B9" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C9" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="5">
         <v>153615616</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D10" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E10" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B10" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C10" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="5">
         <v>197486511</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E11" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B11" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C11" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="5">
         <v>125964931</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E12" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B12" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C12" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="5">
         <v>183572822</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E13" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B13" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C13" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E14" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+        <v>432</v>
+      </c>
+      <c r="B14" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C14" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="5">
         <v>79925209</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E15" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B15" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C15" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="5">
         <v>160931469</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E16" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B16" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C16" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="5">
         <v>144968727</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E17" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B17" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C17" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="5">
         <v>104852513</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E18" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B18" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C18" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="5">
         <v>119864909</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E19" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B19" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C19" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="5">
         <v>91288672</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E20" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B20" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C20" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>434</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E21" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+        <v>433</v>
+      </c>
+      <c r="B21" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C21" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="5">
         <v>124700361</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E22" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B22" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C22" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="5">
         <v>125812759</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E23" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B23" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C23" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>435</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E24" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+        <v>434</v>
+      </c>
+      <c r="B24" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C24" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="5">
         <v>171051738</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E25" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B25" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C25" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>436</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E26" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+        <v>435</v>
+      </c>
+      <c r="B26" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C26" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="5">
         <v>108342544</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E27" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B27" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C27" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="5">
         <v>118830970</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E28" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B28" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C28" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="5">
         <v>154151729</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E29" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B29" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C29" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="5">
         <v>164467473</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E30" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B30" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C30" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="5">
         <v>153616043</v>
       </c>
-      <c r="B31" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E31" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B31" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C31" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>437</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D32" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E32" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+        <v>436</v>
+      </c>
+      <c r="B32" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C32" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="5">
         <v>109199915</v>
       </c>
-      <c r="B33" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E33" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B33" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C33" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="5">
         <v>178129899</v>
       </c>
-      <c r="B34" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D34" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E34" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B34" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C34" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="5">
         <v>156057517</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D35" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E35" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B35" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C35" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="5">
         <v>187493722</v>
       </c>
-      <c r="B36" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D36" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E36" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B36" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C36" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="5">
         <v>163789116</v>
       </c>
-      <c r="B37" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D37" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E37" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B37" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C37" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="5">
         <v>161139238</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D38" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E38" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B38" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C38" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
-        <v>438</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D39" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E39" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+      <c r="B39" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C39" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="5">
         <v>84492795</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D40" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E40" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B40" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C40" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="5">
         <v>200005872</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D41" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E41" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B41" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C41" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="5">
         <v>134408170</v>
       </c>
-      <c r="B42" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D42" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E42" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B42" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C42" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="5">
         <v>77156038</v>
       </c>
-      <c r="B43" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D43" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E43" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B43" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C43" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="5">
         <v>200987489</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D44" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E44" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B44" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C44" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="5">
         <v>83367644</v>
       </c>
-      <c r="B45" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E45" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B45" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C45" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="5">
         <v>186976274</v>
       </c>
-      <c r="B46" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D46" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E46" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B46" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C46" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" s="5">
         <v>105097905</v>
       </c>
-      <c r="B47" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D47" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E47" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B47" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C47" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="5">
         <v>201100895</v>
       </c>
-      <c r="B48" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D48" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E48" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B48" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C48" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="5">
         <v>85760017</v>
       </c>
-      <c r="B49" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D49" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E49" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B49" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C49" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="5">
         <v>100304643</v>
       </c>
-      <c r="B50" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D50" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E50" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B50" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C50" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="5">
         <v>178345036</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D51" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E51" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B51" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C51" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="5">
         <v>176764333</v>
       </c>
-      <c r="B52" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D52" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E52" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B52" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C52" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="5">
         <v>193105610</v>
       </c>
-      <c r="B53" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D53" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E53" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B53" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C53" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="5">
         <v>166217539</v>
       </c>
-      <c r="B54" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D54" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E54" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B54" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C54" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="5">
         <v>188481337</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D55" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E55" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B55" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C55" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="5">
         <v>155407336</v>
       </c>
-      <c r="B56" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D56" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E56" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B56" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C56" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="5">
         <v>172526330</v>
       </c>
-      <c r="B57" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D57" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E57" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B57" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C57" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="5">
         <v>157845322</v>
       </c>
-      <c r="B58" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D58" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E58" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B58" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C58" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="5">
         <v>106451656</v>
       </c>
-      <c r="B59" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D59" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E59" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B59" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C59" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="5">
         <v>227018763</v>
       </c>
-      <c r="B60" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C60" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D60" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E60" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B60" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C60" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" s="5">
         <v>104081665</v>
       </c>
-      <c r="B61" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D61" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E61" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B61" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C61" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" s="5">
         <v>154048219</v>
       </c>
-      <c r="B62" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="C62" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D62" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E62" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B62" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C62" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" s="5">
         <v>186895290</v>
       </c>
-      <c r="B63" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="C63" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D63" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E63" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B63" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C63" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" s="5">
         <v>104368786</v>
       </c>
-      <c r="B64" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="C64" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D64" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E64" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B64" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C64" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="5">
         <v>173059825</v>
       </c>
-      <c r="B65" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="C65" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D65" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E65" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B65" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C65" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" s="5">
         <v>198577278</v>
       </c>
-      <c r="B66" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="C66" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D66" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E66" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B66" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C66" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" s="5">
         <v>155418443</v>
       </c>
-      <c r="B67" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="C67" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D67" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E67" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B67" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C67" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" s="5">
         <v>141203126</v>
       </c>
-      <c r="B68" s="4" t="s">
-        <v>255</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D68" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E68" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B68" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C68" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" s="5">
         <v>156321400</v>
       </c>
-      <c r="B69" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="C69" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D69" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E69" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B69" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C69" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" s="5">
         <v>156095826</v>
       </c>
-      <c r="B70" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="C70" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D70" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E70" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B70" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C70" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" s="5">
         <v>163914476</v>
       </c>
-      <c r="B71" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D71" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E71" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B71" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C71" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
-        <v>439</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="C72" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D72" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E72" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+        <v>438</v>
+      </c>
+      <c r="B72" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C72" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" s="5">
         <v>81135576</v>
       </c>
-      <c r="B73" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="C73" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D73" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E73" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B73" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C73" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" s="5">
         <v>114838454</v>
       </c>
-      <c r="B74" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="C74" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D74" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E74" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B74" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C74" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" s="5">
         <v>134379596</v>
       </c>
-      <c r="B75" s="4" t="s">
-        <v>278</v>
-      </c>
-      <c r="C75" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D75" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E75" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B75" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C75" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" s="5">
         <v>150710162</v>
       </c>
-      <c r="B76" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="C76" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D76" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E76" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B76" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C76" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" s="5">
         <v>164726924</v>
       </c>
-      <c r="B77" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="C77" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D77" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E77" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B77" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C77" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" s="5">
         <v>270091822</v>
       </c>
-      <c r="B78" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D78" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E78" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B78" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C78" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" s="5">
         <v>164110192</v>
       </c>
-      <c r="B79" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D79" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E79" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B79" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C79" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" s="5">
         <v>167419011</v>
       </c>
-      <c r="B80" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="C80" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D80" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E80" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B80" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C80" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" s="5">
         <v>178027255</v>
       </c>
-      <c r="B81" s="4" t="s">
-        <v>296</v>
-      </c>
-      <c r="C81" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D81" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E81" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B81" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C81" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" s="5">
         <v>168035497</v>
       </c>
-      <c r="B82" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="C82" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D82" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E82" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B82" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C82" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" s="5">
         <v>134915013</v>
       </c>
-      <c r="B83" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="C83" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D83" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E83" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B83" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C83" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" s="5">
         <v>124545994</v>
       </c>
-      <c r="B84" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="C84" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D84" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E84" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B84" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C84" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" s="5">
         <v>176778490</v>
       </c>
-      <c r="B85" s="4" t="s">
-        <v>313</v>
-      </c>
-      <c r="C85" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D85" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E85" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B85" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C85" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" s="5">
         <v>182939773</v>
       </c>
-      <c r="B86" s="4" t="s">
-        <v>316</v>
-      </c>
-      <c r="C86" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D86" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E86" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B86" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C86" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" s="5">
         <v>136659995</v>
       </c>
-      <c r="B87" s="4" t="s">
-        <v>319</v>
-      </c>
-      <c r="C87" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D87" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E87" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B87" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C87" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="5">
         <v>122472728</v>
       </c>
-      <c r="B88" s="4" t="s">
-        <v>322</v>
-      </c>
-      <c r="C88" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D88" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E88" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B88" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C88" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" s="5">
         <v>135043060</v>
       </c>
-      <c r="B89" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="C89" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D89" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E89" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B89" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C89" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" s="5">
         <v>163622254</v>
       </c>
-      <c r="B90" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="C90" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D90" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E90" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B90" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C90" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" s="5">
         <v>116777762</v>
       </c>
-      <c r="B91" s="4" t="s">
-        <v>331</v>
-      </c>
-      <c r="C91" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D91" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E91" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B91" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C91" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" s="5">
         <v>162688553</v>
       </c>
-      <c r="B92" s="4" t="s">
-        <v>334</v>
-      </c>
-      <c r="C92" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D92" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E92" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B92" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C92" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" s="5">
         <v>174209391</v>
       </c>
-      <c r="B93" s="4" t="s">
-        <v>337</v>
-      </c>
-      <c r="C93" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D93" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E93" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B93" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C93" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" s="5">
         <v>177084689</v>
       </c>
-      <c r="B94" s="4" t="s">
-        <v>340</v>
-      </c>
-      <c r="C94" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D94" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E94" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B94" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C94" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" s="5">
         <v>120871439</v>
       </c>
-      <c r="B95" s="4" t="s">
-        <v>343</v>
-      </c>
-      <c r="C95" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D95" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E95" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B95" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C95" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" s="5">
         <v>125838138</v>
       </c>
-      <c r="B96" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D96" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E96" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B96" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C96" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" s="5">
         <v>124859964</v>
       </c>
-      <c r="B97" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="C97" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D97" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E97" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B97" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C97" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" s="5">
         <v>129016620</v>
       </c>
-      <c r="B98" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="C98" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D98" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E98" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B98" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C98" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" s="5">
         <v>154654550</v>
       </c>
-      <c r="B99" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="C99" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D99" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E99" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B99" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C99" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A100" s="5">
         <v>204734135</v>
       </c>
-      <c r="B100" s="4" t="s">
-        <v>359</v>
-      </c>
-      <c r="C100" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D100" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E100" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B100" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C100" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" s="5">
         <v>186626907</v>
       </c>
-      <c r="B101" s="4" t="s">
-        <v>368</v>
-      </c>
-      <c r="C101" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D101" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E101" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B101" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C101" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" s="5">
         <v>130922414</v>
       </c>
-      <c r="B102" s="4" t="s">
-        <v>371</v>
-      </c>
-      <c r="C102" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D102" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E102" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B102" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C102" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" s="5">
         <v>169325294</v>
       </c>
-      <c r="B103" s="4" t="s">
-        <v>374</v>
-      </c>
-      <c r="C103" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D103" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E103" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B103" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C103" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" s="5">
         <v>109014494</v>
       </c>
-      <c r="B104" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="C104" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D104" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E104" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B104" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C104" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" s="5">
         <v>105457324</v>
       </c>
-      <c r="B105" s="4" t="s">
-        <v>381</v>
-      </c>
-      <c r="C105" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D105" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E105" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B105" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C105" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" s="5">
         <v>213531492</v>
       </c>
-      <c r="B106" s="4" t="s">
-        <v>384</v>
-      </c>
-      <c r="C106" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D106" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E106" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B106" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C106" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" s="5">
         <v>193752810</v>
       </c>
-      <c r="B107" s="4" t="s">
-        <v>387</v>
-      </c>
-      <c r="C107" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D107" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E107" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B107" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C107" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" s="5">
         <v>156713031</v>
       </c>
-      <c r="B108" s="4" t="s">
-        <v>390</v>
-      </c>
-      <c r="C108" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D108" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E108" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B108" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C108" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" s="5">
         <v>192293197</v>
       </c>
-      <c r="B109" s="4" t="s">
-        <v>393</v>
-      </c>
-      <c r="C109" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D109" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E109" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B109" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C109" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" s="5">
         <v>158701677</v>
       </c>
-      <c r="B110" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="C110" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D110" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E110" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B110" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C110" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" s="5">
         <v>137569701</v>
       </c>
-      <c r="B111" s="4" t="s">
-        <v>399</v>
-      </c>
-      <c r="C111" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D111" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E111" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B111" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C111" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" s="5">
         <v>179298910</v>
       </c>
-      <c r="B112" s="4" t="s">
-        <v>402</v>
-      </c>
-      <c r="C112" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D112" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E112" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B112" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C112" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" s="5">
         <v>89639786</v>
       </c>
-      <c r="B113" s="4" t="s">
-        <v>406</v>
-      </c>
-      <c r="C113" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D113" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E113" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B113" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C113" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" s="5">
         <v>107923896</v>
       </c>
-      <c r="B114" s="4" t="s">
-        <v>410</v>
-      </c>
-      <c r="C114" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D114" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E114" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B114" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C114" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" s="5">
         <v>131394896</v>
       </c>
-      <c r="B115" s="4" t="s">
-        <v>414</v>
-      </c>
-      <c r="C115" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D115" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E115" s="9">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B115" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C115" s="8">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" s="5">
         <v>155892625</v>
       </c>
-      <c r="B116" s="4" t="s">
-        <v>417</v>
-      </c>
-      <c r="C116" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D116" s="9">
-        <v>46122</v>
-      </c>
-      <c r="E116" s="9">
+      <c r="B116" s="8">
+        <v>46122</v>
+      </c>
+      <c r="C116" s="8">
         <v>46295</v>
       </c>
     </row>

</xml_diff>